<commit_message>
fix: texto dos botões no Google Planilhas
Os links entre abas não tinham o atributo display, e o Google Planilhas
mostrava o endereço (#gid=...) no lugar do texto do botão.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AtmR1HynBwWdsg7xxPBTrE
</commit_message>
<xml_diff>
--- a/kit-calculadoras/KIT_6_CALCULADORAS_ENGENHARIA_AMBIENTAL.xlsx
+++ b/kit-calculadoras/KIT_6_CALCULADORAS_ENGENHARIA_AMBIENTAL.xlsx
@@ -3454,16 +3454,16 @@
     <mergeCell ref="B24:D24"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'01 — Comece Aqui'!A1"/>
-    <hyperlink ref="D6" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="F6" location="'01 — Comece Aqui'!B12"/>
-    <hyperlink ref="B13" location="'02 — Vazão e Hidráulica'!A1"/>
-    <hyperlink ref="D13" location="'03 — Carga Poluidora'!A1"/>
-    <hyperlink ref="F13" location="'04 — Eficiência de Tratamento'!A1"/>
-    <hyperlink ref="B20" location="'05 — Balanço de Massa'!A1"/>
-    <hyperlink ref="D20" location="'06 — Diluição de Soluções'!A1"/>
-    <hyperlink ref="F20" location="'07 — Dosagem Química'!A1"/>
-    <hyperlink ref="B29" location="'01 — Comece Aqui'!A1"/>
+    <hyperlink ref="B6" location="'01 — Comece Aqui'!A1" tooltip="Ir para 01 — Comece Aqui" display="📘  COMECE AQUI (GUIA)"/>
+    <hyperlink ref="D6" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="📚  BIBLIOTECA DE EXEMPLOS"/>
+    <hyperlink ref="F6" location="'01 — Comece Aqui'!B12" tooltip="Ir para 01 — Comece Aqui" display="▶  COMO USAR EM 5 PASSOS"/>
+    <hyperlink ref="B13" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="Abrir calculadora  ▶"/>
+    <hyperlink ref="D13" location="'03 — Carga Poluidora'!A1" tooltip="Ir para 03 — Carga Poluidora" display="Abrir calculadora  ▶"/>
+    <hyperlink ref="F13" location="'04 — Eficiência de Tratamento'!A1" tooltip="Ir para 04 — Eficiência de Tratamento" display="Abrir calculadora  ▶"/>
+    <hyperlink ref="B20" location="'05 — Balanço de Massa'!A1" tooltip="Ir para 05 — Balanço de Massa" display="Abrir calculadora  ▶"/>
+    <hyperlink ref="D20" location="'06 — Diluição de Soluções'!A1" tooltip="Ir para 06 — Diluição de Soluções" display="Abrir calculadora  ▶"/>
+    <hyperlink ref="F20" location="'07 — Dosagem Química'!A1" tooltip="Ir para 07 — Dosagem Química" display="Abrir calculadora  ▶"/>
+    <hyperlink ref="B29" location="'01 — Comece Aqui'!A1" tooltip="Ir para 01 — Comece Aqui" display="Dúvidas? Abra o guia completo na aba 01: Comece Aqui."/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
@@ -5081,28 +5081,28 @@
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1"/>
-    <hyperlink ref="C3" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="D3" location="'02 — Vazão e Hidráulica'!A1"/>
-    <hyperlink ref="B21" location="'02 — Vazão e Hidráulica'!A1"/>
-    <hyperlink ref="B22" location="'03 — Carga Poluidora'!A1"/>
-    <hyperlink ref="B23" location="'04 — Eficiência de Tratamento'!A1"/>
-    <hyperlink ref="B24" location="'05 — Balanço de Massa'!A1"/>
-    <hyperlink ref="B25" location="'06 — Diluição de Soluções'!A1"/>
-    <hyperlink ref="B26" location="'07 — Dosagem Química'!A1"/>
-    <hyperlink ref="C30" location="'02 — Vazão e Hidráulica'!A1"/>
-    <hyperlink ref="C31" location="'02 — Vazão e Hidráulica'!A1"/>
-    <hyperlink ref="C32" location="'02 — Vazão e Hidráulica'!A1"/>
-    <hyperlink ref="C33" location="'02 — Vazão e Hidráulica'!A1"/>
-    <hyperlink ref="C34" location="'03 — Carga Poluidora'!A1"/>
-    <hyperlink ref="C35" location="'03 — Carga Poluidora'!A1"/>
-    <hyperlink ref="C36" location="'04 — Eficiência de Tratamento'!A1"/>
-    <hyperlink ref="C37" location="'05 — Balanço de Massa'!A1"/>
-    <hyperlink ref="C38" location="'05 — Balanço de Massa'!A1"/>
-    <hyperlink ref="C39" location="'05 — Balanço de Massa'!A1"/>
-    <hyperlink ref="C40" location="'06 — Diluição de Soluções'!A1"/>
-    <hyperlink ref="C41" location="'07 — Dosagem Química'!A1"/>
-    <hyperlink ref="B122" location="'00 — Painel Inicial'!A1"/>
+    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1" tooltip="Ir para 00 — Painel Inicial" display="🏠  Painel Inicial"/>
+    <hyperlink ref="C3" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="📚  Exemplos Resolvidos"/>
+    <hyperlink ref="D3" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="Primeira calculadora ▶"/>
+    <hyperlink ref="B21" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="💧 01 · Vazão e Hidráulica"/>
+    <hyperlink ref="B22" location="'03 — Carga Poluidora'!A1" tooltip="Ir para 03 — Carga Poluidora" display="🏭 02 · Carga Poluidora"/>
+    <hyperlink ref="B23" location="'04 — Eficiência de Tratamento'!A1" tooltip="Ir para 04 — Eficiência de Tratamento" display="📉 03 · Eficiência"/>
+    <hyperlink ref="B24" location="'05 — Balanço de Massa'!A1" tooltip="Ir para 05 — Balanço de Massa" display="⚖️ 04 · Balanço de Massa"/>
+    <hyperlink ref="B25" location="'06 — Diluição de Soluções'!A1" tooltip="Ir para 06 — Diluição de Soluções" display="🧪 05 · Diluição"/>
+    <hyperlink ref="B26" location="'07 — Dosagem Química'!A1" tooltip="Ir para 07 — Dosagem Química" display="⚗️ 06 · Dosagem Química"/>
+    <hyperlink ref="C30" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="02 · Vazão e Hidráulica (Ferramenta 2)"/>
+    <hyperlink ref="C31" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="02 · Vazão e Hidráulica (Ferramenta 1)"/>
+    <hyperlink ref="C32" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="02 · Vazão e Hidráulica (Ferramenta 3)"/>
+    <hyperlink ref="C33" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="02 · Vazão e Hidráulica (Ferramenta 4)"/>
+    <hyperlink ref="C34" location="'03 — Carga Poluidora'!A1" tooltip="Ir para 03 — Carga Poluidora" display="03 · Carga Poluidora (Ferramenta 1)"/>
+    <hyperlink ref="C35" location="'03 — Carga Poluidora'!A1" tooltip="Ir para 03 — Carga Poluidora" display="03 · Carga Poluidora (Ferramenta 2)"/>
+    <hyperlink ref="C36" location="'04 — Eficiência de Tratamento'!A1" tooltip="Ir para 04 — Eficiência de Tratamento" display="04 · Eficiência de Tratamento"/>
+    <hyperlink ref="C37" location="'05 — Balanço de Massa'!A1" tooltip="Ir para 05 — Balanço de Massa" display="05 · Balanço de Massa (Ferramenta 1)"/>
+    <hyperlink ref="C38" location="'05 — Balanço de Massa'!A1" tooltip="Ir para 05 — Balanço de Massa" display="05 · Balanço de Massa (Ferramenta 2)"/>
+    <hyperlink ref="C39" location="'05 — Balanço de Massa'!A1" tooltip="Ir para 05 — Balanço de Massa" display="05 · Balanço de Massa (Ferramenta 3)"/>
+    <hyperlink ref="C40" location="'06 — Diluição de Soluções'!A1" tooltip="Ir para 06 — Diluição de Soluções" display="06 · Diluição de Soluções"/>
+    <hyperlink ref="C41" location="'07 — Dosagem Química'!A1" tooltip="Ir para 07 — Dosagem Química" display="07 · Dosagem Química"/>
+    <hyperlink ref="B122" location="'00 — Painel Inicial'!A1" tooltip="Ir para 00 — Painel Inicial" display="Tudo pronto?  Voltar ao Painel Inicial e escolher uma calculadora  ▶"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -8889,19 +8889,19 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1"/>
-    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1"/>
-    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G3" location="'01 — Comece Aqui'!A1"/>
-    <hyperlink ref="H3" location="'03 — Carga Poluidora'!A1"/>
-    <hyperlink ref="B13" location="'02 — Vazão e Hidráulica'!B22"/>
-    <hyperlink ref="B14" location="'02 — Vazão e Hidráulica'!B58"/>
-    <hyperlink ref="B15" location="'02 — Vazão e Hidráulica'!B93"/>
-    <hyperlink ref="B16" location="'02 — Vazão e Hidráulica'!B129"/>
-    <hyperlink ref="H22" location="'02 — Vazão e Hidráulica'!A1"/>
-    <hyperlink ref="H58" location="'02 — Vazão e Hidráulica'!A1"/>
-    <hyperlink ref="H93" location="'02 — Vazão e Hidráulica'!A1"/>
-    <hyperlink ref="H129" location="'02 — Vazão e Hidráulica'!A1"/>
+    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1" tooltip="Ir para 00 — Painel Inicial" display="🏠  Painel"/>
+    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1" tooltip="Ir para 01 — Comece Aqui" display="📘  Guia"/>
+    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="📚  Exemplos"/>
+    <hyperlink ref="G3" location="'01 — Comece Aqui'!A1" tooltip="Ir para 01 — Comece Aqui" display="◀ Anterior"/>
+    <hyperlink ref="H3" location="'03 — Carga Poluidora'!A1" tooltip="Ir para 03 — Carga Poluidora" display="Próxima aba ▶"/>
+    <hyperlink ref="B13" location="'02 — Vazão e Hidráulica'!B22" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Ferramenta 1"/>
+    <hyperlink ref="B14" location="'02 — Vazão e Hidráulica'!B58" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Ferramenta 2"/>
+    <hyperlink ref="B15" location="'02 — Vazão e Hidráulica'!B93" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Ferramenta 3"/>
+    <hyperlink ref="B16" location="'02 — Vazão e Hidráulica'!B129" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Ferramenta 4"/>
+    <hyperlink ref="H22" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="▲ Voltar ao topo"/>
+    <hyperlink ref="H58" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="▲ Voltar ao topo"/>
+    <hyperlink ref="H93" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="▲ Voltar ao topo"/>
+    <hyperlink ref="H129" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="▲ Voltar ao topo"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -11660,17 +11660,17 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1"/>
-    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1"/>
-    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G3" location="'02 — Vazão e Hidráulica'!A1"/>
-    <hyperlink ref="H3" location="'04 — Eficiência de Tratamento'!A1"/>
-    <hyperlink ref="B13" location="'03 — Carga Poluidora'!B21"/>
-    <hyperlink ref="B14" location="'03 — Carga Poluidora'!B57"/>
-    <hyperlink ref="B15" location="'03 — Carga Poluidora'!B93"/>
-    <hyperlink ref="H21" location="'03 — Carga Poluidora'!A1"/>
-    <hyperlink ref="H57" location="'03 — Carga Poluidora'!A1"/>
-    <hyperlink ref="H93" location="'03 — Carga Poluidora'!A1"/>
+    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1" tooltip="Ir para 00 — Painel Inicial" display="🏠  Painel"/>
+    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1" tooltip="Ir para 01 — Comece Aqui" display="📘  Guia"/>
+    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="📚  Exemplos"/>
+    <hyperlink ref="G3" location="'02 — Vazão e Hidráulica'!A1" tooltip="Ir para 02 — Vazão e Hidráulica" display="◀ Anterior"/>
+    <hyperlink ref="H3" location="'04 — Eficiência de Tratamento'!A1" tooltip="Ir para 04 — Eficiência de Tratamento" display="Próxima aba ▶"/>
+    <hyperlink ref="B13" location="'03 — Carga Poluidora'!B21" tooltip="Ir para 03 — Carga Poluidora" display="▶ Ferramenta 1"/>
+    <hyperlink ref="B14" location="'03 — Carga Poluidora'!B57" tooltip="Ir para 03 — Carga Poluidora" display="▶ Ferramenta 2"/>
+    <hyperlink ref="B15" location="'03 — Carga Poluidora'!B93" tooltip="Ir para 03 — Carga Poluidora" display="▶ Ferramenta 3"/>
+    <hyperlink ref="H21" location="'03 — Carga Poluidora'!A1" tooltip="Ir para 03 — Carga Poluidora" display="▲ Voltar ao topo"/>
+    <hyperlink ref="H57" location="'03 — Carga Poluidora'!A1" tooltip="Ir para 03 — Carga Poluidora" display="▲ Voltar ao topo"/>
+    <hyperlink ref="H93" location="'03 — Carga Poluidora'!A1" tooltip="Ir para 03 — Carga Poluidora" display="▲ Voltar ao topo"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -13939,15 +13939,15 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1"/>
-    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1"/>
-    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G3" location="'03 — Carga Poluidora'!A1"/>
-    <hyperlink ref="H3" location="'05 — Balanço de Massa'!A1"/>
-    <hyperlink ref="B13" location="'04 — Eficiência de Tratamento'!B20"/>
-    <hyperlink ref="B14" location="'04 — Eficiência de Tratamento'!B72"/>
-    <hyperlink ref="H20" location="'04 — Eficiência de Tratamento'!A1"/>
-    <hyperlink ref="H72" location="'04 — Eficiência de Tratamento'!A1"/>
+    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1" tooltip="Ir para 00 — Painel Inicial" display="🏠  Painel"/>
+    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1" tooltip="Ir para 01 — Comece Aqui" display="📘  Guia"/>
+    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="📚  Exemplos"/>
+    <hyperlink ref="G3" location="'03 — Carga Poluidora'!A1" tooltip="Ir para 03 — Carga Poluidora" display="◀ Anterior"/>
+    <hyperlink ref="H3" location="'05 — Balanço de Massa'!A1" tooltip="Ir para 05 — Balanço de Massa" display="Próxima aba ▶"/>
+    <hyperlink ref="B13" location="'04 — Eficiência de Tratamento'!B20" tooltip="Ir para 04 — Eficiência de Tratamento" display="▶ Ferramenta 1"/>
+    <hyperlink ref="B14" location="'04 — Eficiência de Tratamento'!B72" tooltip="Ir para 04 — Eficiência de Tratamento" display="▶ Ferramenta 2"/>
+    <hyperlink ref="H20" location="'04 — Eficiência de Tratamento'!A1" tooltip="Ir para 04 — Eficiência de Tratamento" display="▲ Voltar ao topo"/>
+    <hyperlink ref="H72" location="'04 — Eficiência de Tratamento'!A1" tooltip="Ir para 04 — Eficiência de Tratamento" display="▲ Voltar ao topo"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -17458,17 +17458,17 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1"/>
-    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1"/>
-    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G3" location="'04 — Eficiência de Tratamento'!A1"/>
-    <hyperlink ref="H3" location="'06 — Diluição de Soluções'!A1"/>
-    <hyperlink ref="B13" location="'05 — Balanço de Massa'!B21"/>
-    <hyperlink ref="B14" location="'05 — Balanço de Massa'!B73"/>
-    <hyperlink ref="B15" location="'05 — Balanço de Massa'!B126"/>
-    <hyperlink ref="H21" location="'05 — Balanço de Massa'!A1"/>
-    <hyperlink ref="H73" location="'05 — Balanço de Massa'!A1"/>
-    <hyperlink ref="H126" location="'05 — Balanço de Massa'!A1"/>
+    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1" tooltip="Ir para 00 — Painel Inicial" display="🏠  Painel"/>
+    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1" tooltip="Ir para 01 — Comece Aqui" display="📘  Guia"/>
+    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="📚  Exemplos"/>
+    <hyperlink ref="G3" location="'04 — Eficiência de Tratamento'!A1" tooltip="Ir para 04 — Eficiência de Tratamento" display="◀ Anterior"/>
+    <hyperlink ref="H3" location="'06 — Diluição de Soluções'!A1" tooltip="Ir para 06 — Diluição de Soluções" display="Próxima aba ▶"/>
+    <hyperlink ref="B13" location="'05 — Balanço de Massa'!B21" tooltip="Ir para 05 — Balanço de Massa" display="▶ Ferramenta 1"/>
+    <hyperlink ref="B14" location="'05 — Balanço de Massa'!B73" tooltip="Ir para 05 — Balanço de Massa" display="▶ Ferramenta 2"/>
+    <hyperlink ref="B15" location="'05 — Balanço de Massa'!B126" tooltip="Ir para 05 — Balanço de Massa" display="▶ Ferramenta 3"/>
+    <hyperlink ref="H21" location="'05 — Balanço de Massa'!A1" tooltip="Ir para 05 — Balanço de Massa" display="▲ Voltar ao topo"/>
+    <hyperlink ref="H73" location="'05 — Balanço de Massa'!A1" tooltip="Ir para 05 — Balanço de Massa" display="▲ Voltar ao topo"/>
+    <hyperlink ref="H126" location="'05 — Balanço de Massa'!A1" tooltip="Ir para 05 — Balanço de Massa" display="▲ Voltar ao topo"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -19292,13 +19292,13 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1"/>
-    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1"/>
-    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G3" location="'05 — Balanço de Massa'!A1"/>
-    <hyperlink ref="H3" location="'07 — Dosagem Química'!A1"/>
-    <hyperlink ref="B13" location="'06 — Diluição de Soluções'!B15"/>
-    <hyperlink ref="H15" location="'06 — Diluição de Soluções'!A1"/>
+    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1" tooltip="Ir para 00 — Painel Inicial" display="🏠  Painel"/>
+    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1" tooltip="Ir para 01 — Comece Aqui" display="📘  Guia"/>
+    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="📚  Exemplos"/>
+    <hyperlink ref="G3" location="'05 — Balanço de Massa'!A1" tooltip="Ir para 05 — Balanço de Massa" display="◀ Anterior"/>
+    <hyperlink ref="H3" location="'07 — Dosagem Química'!A1" tooltip="Ir para 07 — Dosagem Química" display="Próxima aba ▶"/>
+    <hyperlink ref="B13" location="'06 — Diluição de Soluções'!B15" tooltip="Ir para 06 — Diluição de Soluções" display="▶ Ir para o cálculo"/>
+    <hyperlink ref="H15" location="'06 — Diluição de Soluções'!A1" tooltip="Ir para 06 — Diluição de Soluções" display="▲ Voltar ao topo"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -20704,13 +20704,13 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1"/>
-    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1"/>
-    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G3" location="'06 — Diluição de Soluções'!A1"/>
-    <hyperlink ref="H3" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="B13" location="'07 — Dosagem Química'!B15"/>
-    <hyperlink ref="H15" location="'07 — Dosagem Química'!A1"/>
+    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1" tooltip="Ir para 00 — Painel Inicial" display="🏠  Painel"/>
+    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1" tooltip="Ir para 01 — Comece Aqui" display="📘  Guia"/>
+    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="📚  Exemplos"/>
+    <hyperlink ref="G3" location="'06 — Diluição de Soluções'!A1" tooltip="Ir para 06 — Diluição de Soluções" display="◀ Anterior"/>
+    <hyperlink ref="H3" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="Próxima aba ▶"/>
+    <hyperlink ref="B13" location="'07 — Dosagem Química'!B15" tooltip="Ir para 07 — Dosagem Química" display="▶ Ir para o cálculo"/>
+    <hyperlink ref="H15" location="'07 — Dosagem Química'!A1" tooltip="Ir para 07 — Dosagem Química" display="▲ Voltar ao topo"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -32411,51 +32411,51 @@
     <mergeCell ref="C309:H309"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1"/>
-    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1"/>
-    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G3" location="'07 — Dosagem Química'!A1"/>
-    <hyperlink ref="H3" location="'00 — Painel Inicial'!A1"/>
-    <hyperlink ref="B8" location="'08 — Exemplos Resolvidos'!B15"/>
-    <hyperlink ref="B9" location="'08 — Exemplos Resolvidos'!B98"/>
-    <hyperlink ref="B10" location="'08 — Exemplos Resolvidos'!B161"/>
-    <hyperlink ref="B11" location="'08 — Exemplos Resolvidos'!B204"/>
-    <hyperlink ref="B12" location="'08 — Exemplos Resolvidos'!B267"/>
-    <hyperlink ref="B13" location="'08 — Exemplos Resolvidos'!B290"/>
-    <hyperlink ref="H15" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G17" location="'02 — Vazão e Hidráulica'!B22"/>
-    <hyperlink ref="G27" location="'02 — Vazão e Hidráulica'!B22"/>
-    <hyperlink ref="G37" location="'02 — Vazão e Hidráulica'!B58"/>
-    <hyperlink ref="G47" location="'02 — Vazão e Hidráulica'!B58"/>
-    <hyperlink ref="G57" location="'02 — Vazão e Hidráulica'!B93"/>
-    <hyperlink ref="G67" location="'02 — Vazão e Hidráulica'!B93"/>
-    <hyperlink ref="G77" location="'02 — Vazão e Hidráulica'!B129"/>
-    <hyperlink ref="G87" location="'02 — Vazão e Hidráulica'!B129"/>
-    <hyperlink ref="H98" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G100" location="'03 — Carga Poluidora'!B21"/>
-    <hyperlink ref="G110" location="'03 — Carga Poluidora'!B21"/>
-    <hyperlink ref="G120" location="'03 — Carga Poluidora'!B57"/>
-    <hyperlink ref="G130" location="'03 — Carga Poluidora'!B57"/>
-    <hyperlink ref="G140" location="'03 — Carga Poluidora'!B93"/>
-    <hyperlink ref="G150" location="'03 — Carga Poluidora'!B93"/>
-    <hyperlink ref="H161" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G163" location="'04 — Eficiência de Tratamento'!B20"/>
-    <hyperlink ref="G173" location="'04 — Eficiência de Tratamento'!B20"/>
-    <hyperlink ref="G183" location="'04 — Eficiência de Tratamento'!B72"/>
-    <hyperlink ref="G193" location="'04 — Eficiência de Tratamento'!B72"/>
-    <hyperlink ref="H204" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G206" location="'05 — Balanço de Massa'!B21"/>
-    <hyperlink ref="G216" location="'05 — Balanço de Massa'!B21"/>
-    <hyperlink ref="G226" location="'05 — Balanço de Massa'!B73"/>
-    <hyperlink ref="G236" location="'05 — Balanço de Massa'!B73"/>
-    <hyperlink ref="G246" location="'05 — Balanço de Massa'!B126"/>
-    <hyperlink ref="G256" location="'05 — Balanço de Massa'!B126"/>
-    <hyperlink ref="H267" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G269" location="'06 — Diluição de Soluções'!B15"/>
-    <hyperlink ref="G279" location="'06 — Diluição de Soluções'!B15"/>
-    <hyperlink ref="H290" location="'08 — Exemplos Resolvidos'!A1"/>
-    <hyperlink ref="G292" location="'07 — Dosagem Química'!B15"/>
-    <hyperlink ref="G302" location="'07 — Dosagem Química'!B15"/>
+    <hyperlink ref="B3" location="'00 — Painel Inicial'!A1" tooltip="Ir para 00 — Painel Inicial" display="🏠  Painel"/>
+    <hyperlink ref="C3" location="'01 — Comece Aqui'!A1" tooltip="Ir para 01 — Comece Aqui" display="📘  Guia"/>
+    <hyperlink ref="E3" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="📚  Exemplos"/>
+    <hyperlink ref="G3" location="'07 — Dosagem Química'!A1" tooltip="Ir para 07 — Dosagem Química" display="◀ Anterior"/>
+    <hyperlink ref="H3" location="'00 — Painel Inicial'!A1" tooltip="Ir para 00 — Painel Inicial" display="Próxima aba ▶"/>
+    <hyperlink ref="B8" location="'08 — Exemplos Resolvidos'!B15" tooltip="Ir para 08 — Exemplos Resolvidos" display="💧  01 · Vazão e Hidráulica"/>
+    <hyperlink ref="B9" location="'08 — Exemplos Resolvidos'!B98" tooltip="Ir para 08 — Exemplos Resolvidos" display="🏭  02 · Carga Poluidora"/>
+    <hyperlink ref="B10" location="'08 — Exemplos Resolvidos'!B161" tooltip="Ir para 08 — Exemplos Resolvidos" display="📉  03 · Eficiência"/>
+    <hyperlink ref="B11" location="'08 — Exemplos Resolvidos'!B204" tooltip="Ir para 08 — Exemplos Resolvidos" display="⚖️  04 · Balanço de Massa"/>
+    <hyperlink ref="B12" location="'08 — Exemplos Resolvidos'!B267" tooltip="Ir para 08 — Exemplos Resolvidos" display="🧪  05 · Diluição"/>
+    <hyperlink ref="B13" location="'08 — Exemplos Resolvidos'!B290" tooltip="Ir para 08 — Exemplos Resolvidos" display="⚗️  06 · Dosagem Química"/>
+    <hyperlink ref="H15" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="▲ Voltar ao índice"/>
+    <hyperlink ref="G17" location="'02 — Vazão e Hidráulica'!B22" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G27" location="'02 — Vazão e Hidráulica'!B22" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G37" location="'02 — Vazão e Hidráulica'!B58" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G47" location="'02 — Vazão e Hidráulica'!B58" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G57" location="'02 — Vazão e Hidráulica'!B93" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G67" location="'02 — Vazão e Hidráulica'!B93" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G77" location="'02 — Vazão e Hidráulica'!B129" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G87" location="'02 — Vazão e Hidráulica'!B129" tooltip="Ir para 02 — Vazão e Hidráulica" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="H98" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="▲ Voltar ao índice"/>
+    <hyperlink ref="G100" location="'03 — Carga Poluidora'!B21" tooltip="Ir para 03 — Carga Poluidora" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G110" location="'03 — Carga Poluidora'!B21" tooltip="Ir para 03 — Carga Poluidora" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G120" location="'03 — Carga Poluidora'!B57" tooltip="Ir para 03 — Carga Poluidora" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G130" location="'03 — Carga Poluidora'!B57" tooltip="Ir para 03 — Carga Poluidora" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G140" location="'03 — Carga Poluidora'!B93" tooltip="Ir para 03 — Carga Poluidora" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G150" location="'03 — Carga Poluidora'!B93" tooltip="Ir para 03 — Carga Poluidora" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="H161" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="▲ Voltar ao índice"/>
+    <hyperlink ref="G163" location="'04 — Eficiência de Tratamento'!B20" tooltip="Ir para 04 — Eficiência de Tratamento" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G173" location="'04 — Eficiência de Tratamento'!B20" tooltip="Ir para 04 — Eficiência de Tratamento" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G183" location="'04 — Eficiência de Tratamento'!B72" tooltip="Ir para 04 — Eficiência de Tratamento" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G193" location="'04 — Eficiência de Tratamento'!B72" tooltip="Ir para 04 — Eficiência de Tratamento" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="H204" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="▲ Voltar ao índice"/>
+    <hyperlink ref="G206" location="'05 — Balanço de Massa'!B21" tooltip="Ir para 05 — Balanço de Massa" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G216" location="'05 — Balanço de Massa'!B21" tooltip="Ir para 05 — Balanço de Massa" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G226" location="'05 — Balanço de Massa'!B73" tooltip="Ir para 05 — Balanço de Massa" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G236" location="'05 — Balanço de Massa'!B73" tooltip="Ir para 05 — Balanço de Massa" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G246" location="'05 — Balanço de Massa'!B126" tooltip="Ir para 05 — Balanço de Massa" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G256" location="'05 — Balanço de Massa'!B126" tooltip="Ir para 05 — Balanço de Massa" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="H267" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="▲ Voltar ao índice"/>
+    <hyperlink ref="G269" location="'06 — Diluição de Soluções'!B15" tooltip="Ir para 06 — Diluição de Soluções" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G279" location="'06 — Diluição de Soluções'!B15" tooltip="Ir para 06 — Diluição de Soluções" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="H290" location="'08 — Exemplos Resolvidos'!A1" tooltip="Ir para 08 — Exemplos Resolvidos" display="▲ Voltar ao índice"/>
+    <hyperlink ref="G292" location="'07 — Dosagem Química'!B15" tooltip="Ir para 07 — Dosagem Química" display="▶ Abrir na calculadora"/>
+    <hyperlink ref="G302" location="'07 — Dosagem Química'!B15" tooltip="Ir para 07 — Dosagem Química" display="▶ Abrir na calculadora"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>